<commit_message>
Update Portfolio.jsx with new changes
</commit_message>
<xml_diff>
--- a/src/assets/newportfoliodata.xlsx
+++ b/src/assets/newportfoliodata.xlsx
@@ -12,7 +12,6 @@
     <sheet name="Sheet3" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="125725"/>
-  <fileRecoveryPr repairLoad="1"/>
 </workbook>
 </file>
 
@@ -404,7 +403,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I38"/>
+  <dimension ref="A1:I37"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.85546875" customWidth="1"/>
@@ -1107,37 +1106,15 @@
       </c>
     </row>
     <row r="22" spans="1:9">
-      <c r="A22" s="6">
-        <v>45929</v>
-      </c>
-      <c r="B22" s="2">
-        <v>3500</v>
-      </c>
-      <c r="C22" s="3">
-        <f t="shared" ref="C22" si="8">B22/100000*100</f>
-        <v>3.5000000000000004</v>
-      </c>
-      <c r="D22" s="2">
-        <v>3000</v>
-      </c>
-      <c r="E22" s="3">
-        <f t="shared" ref="E22" si="9">D22/100000*100</f>
-        <v>3</v>
-      </c>
-      <c r="F22" s="2">
-        <v>4000</v>
-      </c>
-      <c r="G22" s="3">
-        <f t="shared" ref="G22" si="10">F22/100000*100</f>
-        <v>4</v>
-      </c>
-      <c r="H22" s="2">
-        <v>5550</v>
-      </c>
-      <c r="I22" s="4">
-        <f t="shared" ref="I22" si="11">H22/100000*100</f>
-        <v>5.55</v>
-      </c>
+      <c r="A22" s="5"/>
+      <c r="B22" s="2"/>
+      <c r="C22" s="3"/>
+      <c r="D22" s="2"/>
+      <c r="E22" s="3"/>
+      <c r="F22" s="2"/>
+      <c r="G22" s="3"/>
+      <c r="H22" s="2"/>
+      <c r="I22" s="4"/>
     </row>
     <row r="23" spans="1:9">
       <c r="A23" s="5"/>
@@ -1303,17 +1280,6 @@
       <c r="G37" s="3"/>
       <c r="H37" s="2"/>
       <c r="I37" s="4"/>
-    </row>
-    <row r="38" spans="1:9">
-      <c r="A38" s="5"/>
-      <c r="B38" s="2"/>
-      <c r="C38" s="3"/>
-      <c r="D38" s="2"/>
-      <c r="E38" s="3"/>
-      <c r="F38" s="2"/>
-      <c r="G38" s="3"/>
-      <c r="H38" s="2"/>
-      <c r="I38" s="4"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>